<commit_message>
feat: add duration insights to hackathon infographic
</commit_message>
<xml_diff>
--- a/outputs/linkedin-people-directory/Hackathon CV.xlsx
+++ b/outputs/linkedin-people-directory/Hackathon CV.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hackathons" sheetId="1" r:id="Rc19c9d3b1df04ca2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="People" sheetId="2" r:id="Rbf276a3e885d4d81"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socials" sheetId="3" r:id="R42df29894e6c4d83"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hackathons" sheetId="1" r:id="R2609c21a010947d9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="People" sheetId="2" r:id="Rb9517d237638476e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socials" sheetId="3" r:id="Rc52ba41063f6422f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1687,12 +1687,27 @@
       <x:name val="Calibri"/>
     </x:font>
   </x:fonts>
-  <x:fills count="68">
+  <x:fills count="71">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="gray125"/>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF111111"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF3D5"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF21D2F"/>
+      </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
@@ -2060,7 +2075,7 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="274">
+  <x:cellXfs count="286">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -2579,6 +2594,28 @@
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="4" fillId="67" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="68" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="68" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="68" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="69" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="69" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="69" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="69" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="70" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="70" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="70" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="70" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="70" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -2614,7 +2651,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="31" name="PeopleDirectory" displayName="PeopleDirectory" ref="A4:E97" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="33" name="PeopleDirectory" displayName="PeopleDirectory" ref="A4:E97" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A4:E97"/>
   <x:tableColumns count="5">
     <x:tableColumn id="1" name="Person ID"/>
@@ -2628,7 +2665,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="32" name="HackathonSocials" displayName="HackathonSocials" ref="A4:D78" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="34" name="HackathonSocials" displayName="HackathonSocials" ref="A4:D78" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A4:D78"/>
   <x:tableColumns count="4">
     <x:tableColumn id="1" name="Hackathon #"/>
@@ -6546,8 +6583,8 @@
     </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="R3125aaa772464745"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P61" r:id="Rde171be31a8b4499"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="Rcb015424c2f84c3f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P61" r:id="Rf9b6232306704f25"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -6569,37 +6606,37 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="38" customHeight="1">
-      <x:c r="A1" s="264" t="str">
+      <x:c r="A1" s="276" t="str">
         <x:v>People &amp; LinkedIn Directory</x:v>
       </x:c>
-      <x:c r="B1" s="264"/>
-      <x:c r="C1" s="264"/>
-      <x:c r="D1" s="264"/>
-      <x:c r="E1" s="264"/>
+      <x:c r="B1" s="276"/>
+      <x:c r="C1" s="276"/>
+      <x:c r="D1" s="276"/>
+      <x:c r="E1" s="276"/>
     </x:row>
     <x:row r="2" ht="34" customHeight="1">
-      <x:c r="A2" s="268" t="str">
+      <x:c r="A2" s="280" t="str">
         <x:v>One person per row. LinkedIn URLs are added only after the profile has been verified against the hackathon context.</x:v>
       </x:c>
-      <x:c r="B2" s="268"/>
-      <x:c r="C2" s="268"/>
-      <x:c r="D2" s="268"/>
-      <x:c r="E2" s="268"/>
+      <x:c r="B2" s="280"/>
+      <x:c r="C2" s="280"/>
+      <x:c r="D2" s="280"/>
+      <x:c r="E2" s="280"/>
     </x:row>
     <x:row r="4" ht="30" customHeight="1">
-      <x:c r="A4" s="273" t="str">
+      <x:c r="A4" s="285" t="str">
         <x:v>Person ID</x:v>
       </x:c>
-      <x:c r="B4" s="273" t="str">
+      <x:c r="B4" s="285" t="str">
         <x:v>Name</x:v>
       </x:c>
-      <x:c r="C4" s="273" t="str">
+      <x:c r="C4" s="285" t="str">
         <x:v>Hackathon #s</x:v>
       </x:c>
-      <x:c r="D4" s="273" t="str">
+      <x:c r="D4" s="285" t="str">
         <x:v>Builds Together</x:v>
       </x:c>
-      <x:c r="E4" s="273" t="str">
+      <x:c r="E4" s="285" t="str">
         <x:v>LinkedIn URL</x:v>
       </x:c>
     </x:row>
@@ -8114,12 +8151,12 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="R88f217f5678d49e9"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="Rc5d39091b8554c39"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="R8d7a8f25ddcf4588"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="Rddf8793821f740cb"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra0d479790cd04231"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R42f392b163b24c57"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8135,32 +8172,32 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="38" customHeight="1">
-      <x:c r="A1" s="264" t="str">
+      <x:c r="A1" s="276" t="str">
         <x:v>Socials by Hackathon</x:v>
       </x:c>
-      <x:c r="B1" s="264"/>
-      <x:c r="C1" s="264"/>
-      <x:c r="D1" s="264"/>
+      <x:c r="B1" s="276"/>
+      <x:c r="C1" s="276"/>
+      <x:c r="D1" s="276"/>
     </x:row>
     <x:row r="2" ht="34" customHeight="1">
-      <x:c r="A2" s="268" t="str">
+      <x:c r="A2" s="280" t="str">
         <x:v>One row per numbered hackathon. Add only posts that clearly document the relevant build or event.</x:v>
       </x:c>
-      <x:c r="B2" s="268"/>
-      <x:c r="C2" s="268"/>
-      <x:c r="D2" s="268"/>
+      <x:c r="B2" s="280"/>
+      <x:c r="C2" s="280"/>
+      <x:c r="D2" s="280"/>
     </x:row>
     <x:row r="4" ht="30" customHeight="1">
-      <x:c r="A4" s="273" t="str">
+      <x:c r="A4" s="285" t="str">
         <x:v>Hackathon #</x:v>
       </x:c>
-      <x:c r="B4" s="273" t="str">
+      <x:c r="B4" s="285" t="str">
         <x:v>LinkedIn</x:v>
       </x:c>
-      <x:c r="C4" s="273" t="str">
+      <x:c r="C4" s="285" t="str">
         <x:v>Instagram</x:v>
       </x:c>
-      <x:c r="D4" s="273" t="str">
+      <x:c r="D4" s="285" t="str">
         <x:v>Facebook</x:v>
       </x:c>
     </x:row>
@@ -8483,7 +8520,10 @@
       <x:c r="B44" s="33" t="str">
         <x:v>https://www.linkedin.com/feed/update/urn:li:activity:7373307701516427264/</x:v>
       </x:c>
-      <x:c r="C44" s="33"/>
+      <x:c r="C44" s="33" t="str">
+        <x:v>https://www.instagram.com/reel/DOVLDxsE37O/
+https://www.instagram.com/reel/DOQFqH8kfeT/</x:v>
+      </x:c>
       <x:c r="D44" s="33"/>
     </x:row>
     <x:row r="45" ht="28" customHeight="1">
@@ -8525,7 +8565,9 @@
         <x:v>#045</x:v>
       </x:c>
       <x:c r="B49" s="33"/>
-      <x:c r="C49" s="33"/>
+      <x:c r="C49" s="33" t="str">
+        <x:v>https://www.instagram.com/reel/DQV0xxIk9ab/</x:v>
+      </x:c>
       <x:c r="D49" s="33"/>
     </x:row>
     <x:row r="50" ht="28" customHeight="1">
@@ -8533,7 +8575,9 @@
         <x:v>#046</x:v>
       </x:c>
       <x:c r="B50" s="33"/>
-      <x:c r="C50" s="33"/>
+      <x:c r="C50" s="33" t="str">
+        <x:v>https://www.instagram.com/reel/DQjw5Lik-5m/</x:v>
+      </x:c>
       <x:c r="D50" s="33"/>
     </x:row>
     <x:row r="51" ht="28" customHeight="1">
@@ -8665,7 +8709,9 @@
       <x:c r="B65" s="33" t="str">
         <x:v>https://www.linkedin.com/feed/update/urn:li:activity:7455961388025389056/</x:v>
       </x:c>
-      <x:c r="C65" s="33"/>
+      <x:c r="C65" s="33" t="str">
+        <x:v>https://www.instagram.com/reel/DXykZomTmXD/</x:v>
+      </x:c>
       <x:c r="D65" s="33"/>
     </x:row>
     <x:row r="66" ht="28" customHeight="1">
@@ -8711,7 +8757,10 @@
       <x:c r="B70" s="33" t="str">
         <x:v>https://www.linkedin.com/feed/update/urn:li:activity:7471043781799178240/</x:v>
       </x:c>
-      <x:c r="C70" s="33"/>
+      <x:c r="C70" s="33" t="str">
+        <x:v>https://www.instagram.com/p/DZc1D4HHbmy/
+https://www.instagram.com/p/DZeIbzgRO-n/</x:v>
+      </x:c>
       <x:c r="D70" s="33"/>
     </x:row>
     <x:row r="71" ht="28" customHeight="1">
@@ -8721,7 +8770,10 @@
       <x:c r="B71" s="33" t="str">
         <x:v>https://www.linkedin.com/feed/update/urn:li:activity:7472197868632571905/</x:v>
       </x:c>
-      <x:c r="C71" s="33"/>
+      <x:c r="C71" s="33" t="str">
+        <x:v>https://www.instagram.com/reel/DZom-hVRIRN/
+https://www.instagram.com/reel/DZonQbURE5R/</x:v>
+      </x:c>
       <x:c r="D71" s="33"/>
     </x:row>
     <x:row r="72" ht="28" customHeight="1">
@@ -8731,7 +8783,10 @@
       <x:c r="B72" s="33" t="str">
         <x:v>https://www.linkedin.com/feed/update/urn:li:activity:7480285163512418306/</x:v>
       </x:c>
-      <x:c r="C72" s="33"/>
+      <x:c r="C72" s="33" t="str">
+        <x:v>https://www.instagram.com/p/DZ3itBVzLwN/
+https://www.instagram.com/p/DZ7AtfFndkJ/</x:v>
+      </x:c>
       <x:c r="D72" s="33"/>
     </x:row>
     <x:row r="73" ht="28" customHeight="1">
@@ -8739,7 +8794,9 @@
         <x:v>#069</x:v>
       </x:c>
       <x:c r="B73" s="33"/>
-      <x:c r="C73" s="33"/>
+      <x:c r="C73" s="33" t="str">
+        <x:v>https://www.instagram.com/p/DZ7Wj9anW7x/</x:v>
+      </x:c>
       <x:c r="D73" s="33"/>
     </x:row>
     <x:row r="74" ht="28" customHeight="1">
@@ -8749,7 +8806,10 @@
       <x:c r="B74" s="33" t="str">
         <x:v>https://www.linkedin.com/feed/update/urn:li:activity:7477508615239585792/</x:v>
       </x:c>
-      <x:c r="C74" s="33"/>
+      <x:c r="C74" s="33" t="str">
+        <x:v>https://www.instagram.com/p/DaFSqK7k2ce/
+https://www.instagram.com/reel/DaFm4k2zifY/</x:v>
+      </x:c>
       <x:c r="D74" s="33"/>
     </x:row>
     <x:row r="75" ht="28" customHeight="1">
@@ -8759,7 +8819,9 @@
       <x:c r="B75" s="33" t="str">
         <x:v>https://www.linkedin.com/feed/update/urn:li:activity:7482072463900835840/</x:v>
       </x:c>
-      <x:c r="C75" s="33"/>
+      <x:c r="C75" s="33" t="str">
+        <x:v>https://www.instagram.com/p/Dash2D1k4C2/</x:v>
+      </x:c>
       <x:c r="D75" s="33"/>
     </x:row>
     <x:row r="76" ht="28" customHeight="1">
@@ -8769,7 +8831,11 @@
       <x:c r="B76" s="33" t="str">
         <x:v>https://www.linkedin.com/feed/update/urn:li:activity:7486774772140474368/</x:v>
       </x:c>
-      <x:c r="C76" s="33"/>
+      <x:c r="C76" s="33" t="str">
+        <x:v>https://www.instagram.com/p/DbN5kZlk0LL/
+https://www.instagram.com/reel/DbN4xRaxZY8/
+https://www.instagram.com/reel/DbN5OnlRCGQ/</x:v>
+      </x:c>
       <x:c r="D76" s="33"/>
     </x:row>
     <x:row r="77" ht="28" customHeight="1">
@@ -8777,7 +8843,9 @@
         <x:v>#073</x:v>
       </x:c>
       <x:c r="B77" s="33"/>
-      <x:c r="C77" s="33"/>
+      <x:c r="C77" s="33" t="str">
+        <x:v>https://www.instagram.com/p/DbpmfeiHexb/</x:v>
+      </x:c>
       <x:c r="D77" s="33"/>
     </x:row>
     <x:row r="78" ht="28" customHeight="1">
@@ -8797,7 +8865,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfbcab74682574abe"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc73dcc3c9a6249ac"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>